<commit_message>
feat: add protocol packets and game server updates
- Add new protocol packets: freeze, holyday_screen, item_throw_confirm, ui_screen, unknown_12/1B/26/35/4B/6A, update_cc
- Update character and protocol headers
- Update game server lib: achievement, appearance, character, channels, handlers, items, listeners, marketplace, marriage, models, object, protocol, quest, server, stat
- Update spell table and Lua scripts (mimicry rename, add 정지 spell)
- Update bot tests, fb server, gateway, login server
</commit_message>
<xml_diff>
--- a/resources/table/spell.xlsx
+++ b/resources/table/spell.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F91F49F-E44A-4417-9175-3396BC99589A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4942B40-ECB8-44FB-8B4C-9EB5F14915A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="spell" sheetId="1" r:id="rId1"/>
@@ -3127,12 +3127,6 @@
     <t>14</t>
   </si>
   <si>
-    <t>의태시약</t>
-  </si>
-  <si>
-    <t>scripts/spell/의태시약.lua</t>
-  </si>
-  <si>
     <t>ON_CAST_14</t>
   </si>
   <si>
@@ -3149,12 +3143,6 @@
   </si>
   <si>
     <t>15</t>
-  </si>
-  <si>
-    <t>의태시약10</t>
-  </si>
-  <si>
-    <t>scripts/spell/의태시약10.lua</t>
   </si>
   <si>
     <t>ON_CAST_15</t>
@@ -4512,6 +4500,22 @@
   </si>
   <si>
     <t>scripts/spell/용천제구격.lua</t>
+  </si>
+  <si>
+    <t>의태</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정지</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/spell/정지.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scripts/spell/의태.lua</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -9799,2220 +9803,2220 @@
         <v>1030</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>1031</v>
+        <v>1489</v>
       </c>
       <c r="C219" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D219" s="1" t="s">
+        <v>1492</v>
+      </c>
+      <c r="E219" s="1" t="s">
+        <v>1031</v>
+      </c>
+      <c r="F219" s="1" t="s">
         <v>1032</v>
       </c>
-      <c r="E219" s="1" t="s">
+      <c r="G219" s="1" t="s">
         <v>1033</v>
       </c>
-      <c r="F219" s="1" t="s">
+      <c r="I219" s="1" t="s">
         <v>1034</v>
       </c>
-      <c r="G219" s="1" t="s">
+      <c r="J219" s="1" t="s">
         <v>1035</v>
-      </c>
-      <c r="I219" s="1" t="s">
-        <v>1036</v>
-      </c>
-      <c r="J219" s="1" t="s">
-        <v>1037</v>
       </c>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A220" s="1" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>1039</v>
+        <v>1490</v>
       </c>
       <c r="C220" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D220" s="1" t="s">
-        <v>1040</v>
+        <v>1491</v>
       </c>
       <c r="E220" s="1" t="s">
-        <v>1041</v>
+        <v>1037</v>
       </c>
       <c r="F220" s="1" t="s">
-        <v>1042</v>
+        <v>1038</v>
       </c>
       <c r="G220" s="1" t="s">
-        <v>1043</v>
+        <v>1039</v>
       </c>
       <c r="I220" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J220" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A221" s="1" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="C221" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D221" s="1" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="E221" s="1" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="F221" s="1" t="s">
-        <v>1048</v>
+        <v>1044</v>
       </c>
       <c r="G221" s="1" t="s">
-        <v>1049</v>
+        <v>1045</v>
       </c>
       <c r="I221" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J221" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A222" s="1" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="C222" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D222" s="1" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
       <c r="E222" s="1" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="F222" s="1" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
       <c r="G222" s="1" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="I222" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J222" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A223" s="1" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>1382</v>
+        <v>1378</v>
       </c>
       <c r="C223" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D223" s="1" t="s">
-        <v>1475</v>
+        <v>1471</v>
       </c>
       <c r="E223" s="1" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="F223" s="1" t="s">
-        <v>1060</v>
+        <v>1056</v>
       </c>
       <c r="G223" s="1" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="I223" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J223" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A224" s="1" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>1383</v>
+        <v>1379</v>
       </c>
       <c r="C224" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D224" s="1" t="s">
-        <v>1476</v>
+        <v>1472</v>
       </c>
       <c r="E224" s="1" t="s">
-        <v>1065</v>
+        <v>1061</v>
       </c>
       <c r="F224" s="1" t="s">
-        <v>1066</v>
+        <v>1062</v>
       </c>
       <c r="G224" s="1" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="I224" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J224" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="225" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A225" s="1" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>1384</v>
+        <v>1380</v>
       </c>
       <c r="C225" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D225" s="1" t="s">
-        <v>1477</v>
+        <v>1473</v>
       </c>
       <c r="E225" s="1" t="s">
-        <v>1071</v>
+        <v>1067</v>
       </c>
       <c r="F225" s="1" t="s">
-        <v>1072</v>
+        <v>1068</v>
       </c>
       <c r="G225" s="1" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
       <c r="I225" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J225" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A226" s="1" t="s">
-        <v>1074</v>
+        <v>1070</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>1385</v>
+        <v>1381</v>
       </c>
       <c r="C226" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D226" s="1" t="s">
-        <v>1478</v>
+        <v>1474</v>
       </c>
       <c r="E226" s="1" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
       <c r="F226" s="1" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="G226" s="1" t="s">
-        <v>1079</v>
+        <v>1075</v>
       </c>
       <c r="I226" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J226" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="227" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A227" s="1" t="s">
-        <v>1080</v>
+        <v>1076</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>1386</v>
+        <v>1382</v>
       </c>
       <c r="C227" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D227" s="1" t="s">
-        <v>1479</v>
+        <v>1475</v>
       </c>
       <c r="E227" s="1" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="F227" s="1" t="s">
-        <v>1084</v>
+        <v>1080</v>
       </c>
       <c r="G227" s="1" t="s">
-        <v>1085</v>
+        <v>1081</v>
       </c>
       <c r="I227" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J227" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="228" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A228" s="1" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>1387</v>
+        <v>1383</v>
       </c>
       <c r="C228" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D228" s="1" t="s">
-        <v>1480</v>
+        <v>1476</v>
       </c>
       <c r="E228" s="1" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
       <c r="F228" s="1" t="s">
-        <v>1090</v>
+        <v>1086</v>
       </c>
       <c r="G228" s="1" t="s">
-        <v>1091</v>
+        <v>1087</v>
       </c>
       <c r="I228" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J228" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="229" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A229" s="1" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>1388</v>
+        <v>1384</v>
       </c>
       <c r="C229" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D229" s="1" t="s">
-        <v>1481</v>
+        <v>1477</v>
       </c>
       <c r="E229" s="1" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="F229" s="1" t="s">
-        <v>1096</v>
+        <v>1092</v>
       </c>
       <c r="G229" s="1" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="I229" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J229" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="230" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A230" s="1" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>1389</v>
+        <v>1385</v>
       </c>
       <c r="C230" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D230" s="1" t="s">
-        <v>1482</v>
+        <v>1478</v>
       </c>
       <c r="E230" s="1" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
       <c r="F230" s="1" t="s">
-        <v>1102</v>
+        <v>1098</v>
       </c>
       <c r="G230" s="1" t="s">
-        <v>1103</v>
+        <v>1099</v>
       </c>
       <c r="I230" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J230" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="231" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A231" s="1" t="s">
-        <v>1104</v>
+        <v>1100</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>1390</v>
+        <v>1386</v>
       </c>
       <c r="C231" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D231" s="1" t="s">
-        <v>1483</v>
+        <v>1479</v>
       </c>
       <c r="E231" s="1" t="s">
-        <v>1107</v>
+        <v>1103</v>
       </c>
       <c r="F231" s="1" t="s">
-        <v>1108</v>
+        <v>1104</v>
       </c>
       <c r="G231" s="1" t="s">
-        <v>1109</v>
+        <v>1105</v>
       </c>
       <c r="I231" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J231" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="232" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A232" s="1" t="s">
-        <v>1400</v>
+        <v>1396</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>1391</v>
+        <v>1387</v>
       </c>
       <c r="C232" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D232" s="1" t="s">
-        <v>1484</v>
+        <v>1480</v>
       </c>
       <c r="E232" s="1" t="s">
-        <v>1457</v>
+        <v>1453</v>
       </c>
       <c r="F232" s="1" t="s">
-        <v>1438</v>
+        <v>1434</v>
       </c>
       <c r="G232" s="1" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
       <c r="I232" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J232" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="233" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A233" s="1" t="s">
-        <v>1110</v>
+        <v>1106</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>1392</v>
+        <v>1388</v>
       </c>
       <c r="C233" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D233" s="1" t="s">
-        <v>1485</v>
+        <v>1481</v>
       </c>
       <c r="E233" s="1" t="s">
-        <v>1113</v>
+        <v>1109</v>
       </c>
       <c r="F233" s="1" t="s">
-        <v>1114</v>
+        <v>1110</v>
       </c>
       <c r="G233" s="1" t="s">
-        <v>1115</v>
+        <v>1111</v>
       </c>
       <c r="I233" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J233" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="234" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A234" s="1" t="s">
-        <v>1116</v>
+        <v>1112</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>1393</v>
+        <v>1389</v>
       </c>
       <c r="C234" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D234" s="1" t="s">
-        <v>1486</v>
+        <v>1482</v>
       </c>
       <c r="E234" s="1" t="s">
-        <v>1119</v>
+        <v>1115</v>
       </c>
       <c r="F234" s="1" t="s">
-        <v>1120</v>
+        <v>1116</v>
       </c>
       <c r="G234" s="1" t="s">
-        <v>1121</v>
+        <v>1117</v>
       </c>
       <c r="I234" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J234" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="235" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A235" s="1" t="s">
-        <v>1122</v>
+        <v>1118</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>1394</v>
+        <v>1390</v>
       </c>
       <c r="C235" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D235" s="1" t="s">
-        <v>1487</v>
+        <v>1483</v>
       </c>
       <c r="E235" s="1" t="s">
-        <v>1125</v>
+        <v>1121</v>
       </c>
       <c r="F235" s="1" t="s">
-        <v>1126</v>
+        <v>1122</v>
       </c>
       <c r="G235" s="1" t="s">
-        <v>1127</v>
+        <v>1123</v>
       </c>
       <c r="I235" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J235" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="236" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A236" s="1" t="s">
-        <v>1128</v>
+        <v>1124</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>1395</v>
+        <v>1391</v>
       </c>
       <c r="C236" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D236" s="1" t="s">
-        <v>1488</v>
+        <v>1484</v>
       </c>
       <c r="E236" s="1" t="s">
-        <v>1131</v>
+        <v>1127</v>
       </c>
       <c r="F236" s="1" t="s">
-        <v>1132</v>
+        <v>1128</v>
       </c>
       <c r="G236" s="1" t="s">
-        <v>1133</v>
+        <v>1129</v>
       </c>
       <c r="I236" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J236" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="237" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A237" s="1" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>1396</v>
+        <v>1392</v>
       </c>
       <c r="C237" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D237" s="1" t="s">
-        <v>1489</v>
+        <v>1485</v>
       </c>
       <c r="E237" s="1" t="s">
-        <v>1137</v>
+        <v>1133</v>
       </c>
       <c r="F237" s="1" t="s">
-        <v>1138</v>
+        <v>1134</v>
       </c>
       <c r="G237" s="1" t="s">
-        <v>1139</v>
+        <v>1135</v>
       </c>
       <c r="I237" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J237" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="238" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A238" s="1" t="s">
-        <v>1140</v>
+        <v>1136</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>1397</v>
+        <v>1393</v>
       </c>
       <c r="C238" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D238" s="1" t="s">
-        <v>1490</v>
+        <v>1486</v>
       </c>
       <c r="E238" s="1" t="s">
-        <v>1143</v>
+        <v>1139</v>
       </c>
       <c r="F238" s="1" t="s">
-        <v>1144</v>
+        <v>1140</v>
       </c>
       <c r="G238" s="1" t="s">
-        <v>1145</v>
+        <v>1141</v>
       </c>
       <c r="I238" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J238" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A239" s="1" t="s">
-        <v>1146</v>
+        <v>1142</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>1398</v>
+        <v>1394</v>
       </c>
       <c r="C239" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D239" s="1" t="s">
-        <v>1491</v>
+        <v>1487</v>
       </c>
       <c r="E239" s="1" t="s">
-        <v>1149</v>
+        <v>1145</v>
       </c>
       <c r="F239" s="1" t="s">
-        <v>1150</v>
+        <v>1146</v>
       </c>
       <c r="G239" s="1" t="s">
-        <v>1151</v>
+        <v>1147</v>
       </c>
       <c r="I239" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J239" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="240" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A240" s="1" t="s">
-        <v>1152</v>
+        <v>1148</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>1399</v>
+        <v>1395</v>
       </c>
       <c r="C240" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D240" s="1" t="s">
-        <v>1492</v>
+        <v>1488</v>
       </c>
       <c r="E240" s="1" t="s">
-        <v>1155</v>
+        <v>1151</v>
       </c>
       <c r="F240" s="1" t="s">
-        <v>1156</v>
+        <v>1152</v>
       </c>
       <c r="G240" s="1" t="s">
-        <v>1157</v>
+        <v>1153</v>
       </c>
       <c r="I240" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J240" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="241" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A241" s="1" t="s">
-        <v>1158</v>
+        <v>1154</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="C241" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D241" s="1" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
       <c r="E241" s="1" t="s">
-        <v>1161</v>
+        <v>1157</v>
       </c>
       <c r="F241" s="1" t="s">
-        <v>1162</v>
+        <v>1158</v>
       </c>
       <c r="G241" s="1" t="s">
-        <v>1163</v>
+        <v>1159</v>
       </c>
       <c r="I241" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J241" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="242" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A242" s="1" t="s">
-        <v>1401</v>
+        <v>1397</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>1063</v>
+        <v>1059</v>
       </c>
       <c r="C242" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D242" s="1" t="s">
-        <v>1064</v>
+        <v>1060</v>
       </c>
       <c r="E242" s="1" t="s">
-        <v>1458</v>
+        <v>1454</v>
       </c>
       <c r="F242" s="1" t="s">
-        <v>1439</v>
+        <v>1435</v>
       </c>
       <c r="G242" s="1" t="s">
-        <v>1421</v>
+        <v>1417</v>
       </c>
       <c r="I242" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J242" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A243" s="1" t="s">
-        <v>1402</v>
+        <v>1398</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>1069</v>
+        <v>1065</v>
       </c>
       <c r="C243" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D243" s="1" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="E243" s="1" t="s">
-        <v>1459</v>
+        <v>1455</v>
       </c>
       <c r="F243" s="1" t="s">
-        <v>1440</v>
+        <v>1436</v>
       </c>
       <c r="G243" s="1" t="s">
-        <v>1422</v>
+        <v>1418</v>
       </c>
       <c r="I243" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J243" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="244" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A244" s="1" t="s">
-        <v>1403</v>
+        <v>1399</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>1075</v>
+        <v>1071</v>
       </c>
       <c r="C244" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D244" s="1" t="s">
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="E244" s="1" t="s">
-        <v>1460</v>
+        <v>1456</v>
       </c>
       <c r="F244" s="1" t="s">
-        <v>1441</v>
+        <v>1437</v>
       </c>
       <c r="G244" s="1" t="s">
-        <v>1423</v>
+        <v>1419</v>
       </c>
       <c r="I244" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J244" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A245" s="1" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>1081</v>
+        <v>1077</v>
       </c>
       <c r="C245" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D245" s="1" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="E245" s="1" t="s">
-        <v>1461</v>
+        <v>1457</v>
       </c>
       <c r="F245" s="1" t="s">
-        <v>1442</v>
+        <v>1438</v>
       </c>
       <c r="G245" s="1" t="s">
-        <v>1424</v>
+        <v>1420</v>
       </c>
       <c r="I245" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J245" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A246" s="1" t="s">
-        <v>1405</v>
+        <v>1401</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>1087</v>
+        <v>1083</v>
       </c>
       <c r="C246" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D246" s="1" t="s">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="E246" s="1" t="s">
-        <v>1462</v>
+        <v>1458</v>
       </c>
       <c r="F246" s="1" t="s">
-        <v>1443</v>
+        <v>1439</v>
       </c>
       <c r="G246" s="1" t="s">
-        <v>1425</v>
+        <v>1421</v>
       </c>
       <c r="I246" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J246" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="247" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A247" s="1" t="s">
-        <v>1406</v>
+        <v>1402</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
       <c r="C247" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D247" s="1" t="s">
-        <v>1094</v>
+        <v>1090</v>
       </c>
       <c r="E247" s="1" t="s">
-        <v>1463</v>
+        <v>1459</v>
       </c>
       <c r="F247" s="1" t="s">
-        <v>1444</v>
+        <v>1440</v>
       </c>
       <c r="G247" s="1" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="I247" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J247" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A248" s="1" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>1099</v>
+        <v>1095</v>
       </c>
       <c r="C248" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D248" s="1" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="E248" s="1" t="s">
-        <v>1464</v>
+        <v>1460</v>
       </c>
       <c r="F248" s="1" t="s">
-        <v>1445</v>
+        <v>1441</v>
       </c>
       <c r="G248" s="1" t="s">
-        <v>1427</v>
+        <v>1423</v>
       </c>
       <c r="I248" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J248" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A249" s="1" t="s">
-        <v>1408</v>
+        <v>1404</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>1105</v>
+        <v>1101</v>
       </c>
       <c r="C249" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D249" s="1" t="s">
-        <v>1106</v>
+        <v>1102</v>
       </c>
       <c r="E249" s="1" t="s">
-        <v>1465</v>
+        <v>1461</v>
       </c>
       <c r="F249" s="1" t="s">
-        <v>1446</v>
+        <v>1442</v>
       </c>
       <c r="G249" s="1" t="s">
-        <v>1428</v>
+        <v>1424</v>
       </c>
       <c r="I249" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J249" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="250" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A250" s="1" t="s">
-        <v>1409</v>
+        <v>1405</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>1111</v>
+        <v>1107</v>
       </c>
       <c r="C250" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D250" s="1" t="s">
-        <v>1112</v>
+        <v>1108</v>
       </c>
       <c r="E250" s="1" t="s">
-        <v>1466</v>
+        <v>1462</v>
       </c>
       <c r="F250" s="1" t="s">
-        <v>1447</v>
+        <v>1443</v>
       </c>
       <c r="G250" s="1" t="s">
-        <v>1429</v>
+        <v>1425</v>
       </c>
       <c r="I250" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J250" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A251" s="1" t="s">
-        <v>1410</v>
+        <v>1406</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>1117</v>
+        <v>1113</v>
       </c>
       <c r="C251" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D251" s="1" t="s">
-        <v>1118</v>
+        <v>1114</v>
       </c>
       <c r="E251" s="1" t="s">
-        <v>1467</v>
+        <v>1463</v>
       </c>
       <c r="F251" s="1" t="s">
-        <v>1448</v>
+        <v>1444</v>
       </c>
       <c r="G251" s="1" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="I251" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J251" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="252" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A252" s="1" t="s">
-        <v>1164</v>
+        <v>1160</v>
       </c>
       <c r="B252" s="1" t="s">
-        <v>1123</v>
+        <v>1119</v>
       </c>
       <c r="C252" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D252" s="1" t="s">
-        <v>1124</v>
+        <v>1120</v>
       </c>
       <c r="E252" s="1" t="s">
-        <v>1167</v>
+        <v>1163</v>
       </c>
       <c r="F252" s="1" t="s">
-        <v>1168</v>
+        <v>1164</v>
       </c>
       <c r="G252" s="1" t="s">
-        <v>1169</v>
+        <v>1165</v>
       </c>
       <c r="I252" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J252" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A253" s="1" t="s">
-        <v>1411</v>
+        <v>1407</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>1129</v>
+        <v>1125</v>
       </c>
       <c r="C253" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D253" s="1" t="s">
-        <v>1130</v>
+        <v>1126</v>
       </c>
       <c r="E253" s="1" t="s">
-        <v>1468</v>
+        <v>1464</v>
       </c>
       <c r="F253" s="1" t="s">
-        <v>1449</v>
+        <v>1445</v>
       </c>
       <c r="G253" s="1" t="s">
-        <v>1431</v>
+        <v>1427</v>
       </c>
       <c r="I253" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J253" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A254" s="1" t="s">
-        <v>1412</v>
+        <v>1408</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>1135</v>
+        <v>1131</v>
       </c>
       <c r="C254" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D254" s="1" t="s">
-        <v>1136</v>
+        <v>1132</v>
       </c>
       <c r="E254" s="1" t="s">
-        <v>1469</v>
+        <v>1465</v>
       </c>
       <c r="F254" s="1" t="s">
-        <v>1450</v>
+        <v>1446</v>
       </c>
       <c r="G254" s="1" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="I254" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J254" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A255" s="1" t="s">
-        <v>1170</v>
+        <v>1166</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>1141</v>
+        <v>1137</v>
       </c>
       <c r="C255" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D255" s="1" t="s">
-        <v>1142</v>
+        <v>1138</v>
       </c>
       <c r="E255" s="1" t="s">
-        <v>1173</v>
+        <v>1169</v>
       </c>
       <c r="F255" s="1" t="s">
-        <v>1174</v>
+        <v>1170</v>
       </c>
       <c r="G255" s="1" t="s">
-        <v>1175</v>
+        <v>1171</v>
       </c>
       <c r="I255" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J255" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="256" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A256" s="1" t="s">
-        <v>1413</v>
+        <v>1409</v>
       </c>
       <c r="B256" s="1" t="s">
-        <v>1147</v>
+        <v>1143</v>
       </c>
       <c r="C256" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D256" s="1" t="s">
-        <v>1148</v>
+        <v>1144</v>
       </c>
       <c r="E256" s="1" t="s">
-        <v>1470</v>
+        <v>1466</v>
       </c>
       <c r="F256" s="1" t="s">
-        <v>1451</v>
+        <v>1447</v>
       </c>
       <c r="G256" s="1" t="s">
-        <v>1433</v>
+        <v>1429</v>
       </c>
       <c r="I256" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J256" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="257" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A257" s="1" t="s">
-        <v>1414</v>
+        <v>1410</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>1153</v>
+        <v>1149</v>
       </c>
       <c r="C257" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D257" s="1" t="s">
-        <v>1154</v>
+        <v>1150</v>
       </c>
       <c r="E257" s="1" t="s">
-        <v>1471</v>
+        <v>1467</v>
       </c>
       <c r="F257" s="1" t="s">
-        <v>1452</v>
+        <v>1448</v>
       </c>
       <c r="G257" s="1" t="s">
-        <v>1434</v>
+        <v>1430</v>
       </c>
       <c r="I257" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J257" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="258" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A258" s="1" t="s">
-        <v>1415</v>
+        <v>1411</v>
       </c>
       <c r="B258" s="1" t="s">
-        <v>1159</v>
+        <v>1155</v>
       </c>
       <c r="C258" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D258" s="1" t="s">
-        <v>1160</v>
+        <v>1156</v>
       </c>
       <c r="E258" s="1" t="s">
-        <v>1472</v>
+        <v>1468</v>
       </c>
       <c r="F258" s="1" t="s">
-        <v>1453</v>
+        <v>1449</v>
       </c>
       <c r="G258" s="1" t="s">
-        <v>1435</v>
+        <v>1431</v>
       </c>
       <c r="I258" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J258" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A259" s="1" t="s">
-        <v>1416</v>
+        <v>1412</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>1165</v>
+        <v>1161</v>
       </c>
       <c r="C259" s="1" t="s">
         <v>640</v>
       </c>
       <c r="D259" s="1" t="s">
-        <v>1166</v>
+        <v>1162</v>
       </c>
       <c r="E259" s="1" t="s">
-        <v>1473</v>
+        <v>1469</v>
       </c>
       <c r="F259" s="1" t="s">
-        <v>1454</v>
+        <v>1450</v>
       </c>
       <c r="G259" s="1" t="s">
-        <v>1436</v>
+        <v>1432</v>
       </c>
       <c r="J259" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A260" s="1" t="s">
-        <v>1417</v>
+        <v>1413</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>1171</v>
+        <v>1167</v>
       </c>
       <c r="C260" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D260" s="1" t="s">
-        <v>1172</v>
+        <v>1168</v>
       </c>
       <c r="E260" s="1" t="s">
-        <v>1474</v>
+        <v>1470</v>
       </c>
       <c r="F260" s="1" t="s">
-        <v>1455</v>
+        <v>1451</v>
       </c>
       <c r="G260" s="1" t="s">
-        <v>1437</v>
+        <v>1433</v>
       </c>
       <c r="H260" s="1" t="s">
-        <v>1456</v>
+        <v>1452</v>
       </c>
       <c r="I260" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J260" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A261" s="1" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C261" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="D261" s="1" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E261" s="1" t="s">
+        <v>1175</v>
+      </c>
+      <c r="F261" s="1" t="s">
         <v>1176</v>
       </c>
-      <c r="B261" s="1" t="s">
+      <c r="G261" s="1" t="s">
         <v>1177</v>
       </c>
-      <c r="C261" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="D261" s="1" t="s">
-        <v>1178</v>
-      </c>
-      <c r="E261" s="1" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F261" s="1" t="s">
-        <v>1180</v>
-      </c>
-      <c r="G261" s="1" t="s">
-        <v>1181</v>
-      </c>
       <c r="J261" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="262" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A262" s="1" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C262" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="D262" s="1" t="s">
+        <v>1180</v>
+      </c>
+      <c r="E262" s="1" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F262" s="1" t="s">
         <v>1182</v>
       </c>
-      <c r="B262" s="1" t="s">
+      <c r="G262" s="1" t="s">
         <v>1183</v>
       </c>
-      <c r="C262" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="D262" s="1" t="s">
-        <v>1184</v>
-      </c>
-      <c r="E262" s="1" t="s">
-        <v>1185</v>
-      </c>
-      <c r="F262" s="1" t="s">
-        <v>1186</v>
-      </c>
-      <c r="G262" s="1" t="s">
-        <v>1187</v>
-      </c>
       <c r="J262" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="263" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A263" s="1" t="s">
-        <v>1188</v>
+        <v>1184</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>1189</v>
+        <v>1185</v>
       </c>
       <c r="C263" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D263" s="1" t="s">
-        <v>1190</v>
+        <v>1186</v>
       </c>
       <c r="E263" s="1" t="s">
-        <v>1191</v>
+        <v>1187</v>
       </c>
       <c r="I263" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J263" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A264" s="1" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B264" s="1" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C264" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="D264" s="1" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E264" s="1" t="s">
+        <v>1191</v>
+      </c>
+      <c r="F264" s="1" t="s">
         <v>1192</v>
       </c>
-      <c r="B264" s="1" t="s">
+      <c r="G264" s="1" t="s">
         <v>1193</v>
       </c>
-      <c r="C264" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="D264" s="1" t="s">
+      <c r="H264" s="1" t="s">
         <v>1194</v>
       </c>
-      <c r="E264" s="1" t="s">
-        <v>1195</v>
-      </c>
-      <c r="F264" s="1" t="s">
-        <v>1196</v>
-      </c>
-      <c r="G264" s="1" t="s">
-        <v>1197</v>
-      </c>
-      <c r="H264" s="1" t="s">
-        <v>1198</v>
-      </c>
       <c r="J264" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="265" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A265" s="1" t="s">
-        <v>1418</v>
+        <v>1414</v>
       </c>
       <c r="B265" s="1" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C265" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="D265" s="1" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E265" s="1" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F265" s="1" t="s">
+        <v>1198</v>
+      </c>
+      <c r="G265" s="1" t="s">
         <v>1199</v>
       </c>
-      <c r="C265" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="D265" s="1" t="s">
+      <c r="H265" s="1" t="s">
         <v>1200</v>
       </c>
-      <c r="E265" s="1" t="s">
-        <v>1201</v>
-      </c>
-      <c r="F265" s="1" t="s">
-        <v>1202</v>
-      </c>
-      <c r="G265" s="1" t="s">
-        <v>1203</v>
-      </c>
-      <c r="H265" s="1" t="s">
-        <v>1204</v>
-      </c>
       <c r="J265" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A266" s="1" t="s">
-        <v>1419</v>
+        <v>1415</v>
       </c>
       <c r="B266" s="1" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C266" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="D266" s="1" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E266" s="1" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F266" s="1" t="s">
+        <v>1204</v>
+      </c>
+      <c r="G266" s="1" t="s">
         <v>1205</v>
       </c>
-      <c r="C266" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="D266" s="1" t="s">
+      <c r="H266" s="1" t="s">
         <v>1206</v>
       </c>
-      <c r="E266" s="1" t="s">
-        <v>1207</v>
-      </c>
-      <c r="F266" s="1" t="s">
-        <v>1208</v>
-      </c>
-      <c r="G266" s="1" t="s">
-        <v>1209</v>
-      </c>
-      <c r="H266" s="1" t="s">
-        <v>1210</v>
-      </c>
       <c r="J266" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A267" s="1" t="s">
-        <v>1211</v>
+        <v>1207</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>1212</v>
+        <v>1208</v>
       </c>
       <c r="C267" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D267" s="1" t="s">
-        <v>1213</v>
+        <v>1209</v>
       </c>
       <c r="E267" s="1" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="J267" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A268" s="1" t="s">
-        <v>1215</v>
+        <v>1211</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>1216</v>
+        <v>1212</v>
       </c>
       <c r="C268" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D268" s="1" t="s">
-        <v>1217</v>
+        <v>1213</v>
       </c>
       <c r="E268" s="1" t="s">
-        <v>1218</v>
+        <v>1214</v>
       </c>
       <c r="I268" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J268" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A269" s="1" t="s">
-        <v>1219</v>
+        <v>1215</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>1220</v>
+        <v>1216</v>
       </c>
       <c r="C269" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D269" s="1" t="s">
-        <v>1221</v>
+        <v>1217</v>
       </c>
       <c r="E269" s="1" t="s">
-        <v>1222</v>
+        <v>1218</v>
       </c>
       <c r="I269" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J269" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A270" s="1" t="s">
-        <v>1223</v>
+        <v>1219</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>1224</v>
+        <v>1220</v>
       </c>
       <c r="C270" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D270" s="1" t="s">
-        <v>1225</v>
+        <v>1221</v>
       </c>
       <c r="E270" s="1" t="s">
-        <v>1226</v>
+        <v>1222</v>
       </c>
       <c r="I270" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J270" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="271" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A271" s="1" t="s">
-        <v>1227</v>
+        <v>1223</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>1228</v>
+        <v>1224</v>
       </c>
       <c r="C271" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D271" s="1" t="s">
-        <v>1229</v>
+        <v>1225</v>
       </c>
       <c r="E271" s="1" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
       <c r="I271" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J271" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A272" s="1" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
       <c r="B272" s="1" t="s">
-        <v>1232</v>
+        <v>1228</v>
       </c>
       <c r="C272" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D272" s="1" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="E272" s="1" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
       <c r="I272" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J272" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="273" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A273" s="1" t="s">
-        <v>1235</v>
+        <v>1231</v>
       </c>
       <c r="B273" s="1" t="s">
-        <v>1236</v>
+        <v>1232</v>
       </c>
       <c r="C273" s="1" t="s">
         <v>640</v>
       </c>
       <c r="D273" s="1" t="s">
-        <v>1237</v>
+        <v>1233</v>
       </c>
       <c r="E273" s="1" t="s">
-        <v>1238</v>
+        <v>1234</v>
       </c>
       <c r="J273" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A274" s="1" t="s">
-        <v>1239</v>
+        <v>1235</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>1240</v>
+        <v>1236</v>
       </c>
       <c r="C274" s="1" t="s">
         <v>640</v>
       </c>
       <c r="D274" s="1" t="s">
-        <v>1241</v>
+        <v>1237</v>
       </c>
       <c r="E274" s="1" t="s">
-        <v>1242</v>
+        <v>1238</v>
       </c>
       <c r="J274" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A275" s="1" t="s">
-        <v>1243</v>
+        <v>1239</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>1244</v>
+        <v>1240</v>
       </c>
       <c r="C275" s="1" t="s">
         <v>640</v>
       </c>
       <c r="D275" s="1" t="s">
-        <v>1245</v>
+        <v>1241</v>
       </c>
       <c r="E275" s="1" t="s">
-        <v>1246</v>
+        <v>1242</v>
       </c>
       <c r="J275" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A276" s="1" t="s">
-        <v>1247</v>
+        <v>1243</v>
       </c>
       <c r="B276" s="1" t="s">
-        <v>1248</v>
+        <v>1244</v>
       </c>
       <c r="C276" s="1" t="s">
         <v>640</v>
       </c>
       <c r="D276" s="1" t="s">
-        <v>1249</v>
+        <v>1245</v>
       </c>
       <c r="E276" s="1" t="s">
-        <v>1250</v>
+        <v>1246</v>
       </c>
       <c r="J276" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="277" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A277" s="1" t="s">
-        <v>1251</v>
+        <v>1247</v>
       </c>
       <c r="B277" s="1" t="s">
-        <v>1252</v>
+        <v>1248</v>
       </c>
       <c r="C277" s="1" t="s">
         <v>640</v>
       </c>
       <c r="D277" s="1" t="s">
-        <v>1253</v>
+        <v>1249</v>
       </c>
       <c r="E277" s="1" t="s">
-        <v>1254</v>
+        <v>1250</v>
       </c>
       <c r="J277" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="278" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A278" s="1" t="s">
-        <v>1255</v>
+        <v>1251</v>
       </c>
       <c r="B278" s="1" t="s">
-        <v>1256</v>
+        <v>1252</v>
       </c>
       <c r="C278" s="1" t="s">
         <v>640</v>
       </c>
       <c r="D278" s="1" t="s">
-        <v>1257</v>
+        <v>1253</v>
       </c>
       <c r="E278" s="1" t="s">
-        <v>1258</v>
+        <v>1254</v>
       </c>
       <c r="J278" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="279" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A279" s="1" t="s">
-        <v>1259</v>
+        <v>1255</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>1260</v>
+        <v>1256</v>
       </c>
       <c r="C279" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D279" s="1" t="s">
-        <v>1261</v>
+        <v>1257</v>
       </c>
       <c r="E279" s="1" t="s">
-        <v>1262</v>
+        <v>1258</v>
       </c>
       <c r="I279" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J279" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="280" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A280" s="1" t="s">
-        <v>1263</v>
+        <v>1259</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>1264</v>
+        <v>1260</v>
       </c>
       <c r="C280" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D280" s="1" t="s">
-        <v>1265</v>
+        <v>1261</v>
       </c>
       <c r="E280" s="1" t="s">
-        <v>1266</v>
+        <v>1262</v>
       </c>
       <c r="I280" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J280" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="281" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A281" s="1" t="s">
-        <v>1267</v>
+        <v>1263</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>1268</v>
+        <v>1264</v>
       </c>
       <c r="C281" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D281" s="1" t="s">
-        <v>1269</v>
+        <v>1265</v>
       </c>
       <c r="E281" s="1" t="s">
-        <v>1270</v>
+        <v>1266</v>
       </c>
       <c r="I281" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J281" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="282" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A282" s="1" t="s">
-        <v>1271</v>
+        <v>1267</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>1272</v>
+        <v>1268</v>
       </c>
       <c r="C282" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D282" s="1" t="s">
-        <v>1273</v>
+        <v>1269</v>
       </c>
       <c r="E282" s="1" t="s">
-        <v>1274</v>
+        <v>1270</v>
       </c>
       <c r="I282" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J282" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="283" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A283" s="1" t="s">
-        <v>1275</v>
+        <v>1271</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>1276</v>
+        <v>1272</v>
       </c>
       <c r="C283" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D283" s="1" t="s">
-        <v>1277</v>
+        <v>1273</v>
       </c>
       <c r="E283" s="1" t="s">
-        <v>1278</v>
+        <v>1274</v>
       </c>
       <c r="I283" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J283" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="284" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A284" s="1" t="s">
-        <v>1279</v>
+        <v>1275</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>1280</v>
+        <v>1276</v>
       </c>
       <c r="C284" s="1" t="s">
         <v>641</v>
       </c>
       <c r="D284" s="1" t="s">
-        <v>1281</v>
+        <v>1277</v>
       </c>
       <c r="E284" s="1" t="s">
-        <v>1282</v>
+        <v>1278</v>
       </c>
       <c r="I284" s="1" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="J284" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="285" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A285" s="1" t="s">
-        <v>1283</v>
+        <v>1279</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>1284</v>
+        <v>1280</v>
       </c>
       <c r="C285" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D285" s="1" t="s">
+        <v>1281</v>
+      </c>
+      <c r="E285" s="1" t="s">
+        <v>1282</v>
+      </c>
+      <c r="F285" s="1" t="s">
+        <v>1283</v>
+      </c>
+      <c r="G285" s="1" t="s">
+        <v>1284</v>
+      </c>
+      <c r="H285" s="1" t="s">
         <v>1285</v>
       </c>
-      <c r="E285" s="1" t="s">
+      <c r="I285" s="1" t="s">
         <v>1286</v>
       </c>
-      <c r="F285" s="1" t="s">
-        <v>1287</v>
-      </c>
-      <c r="G285" s="1" t="s">
-        <v>1288</v>
-      </c>
-      <c r="H285" s="1" t="s">
-        <v>1289</v>
-      </c>
-      <c r="I285" s="1" t="s">
-        <v>1290</v>
-      </c>
       <c r="J285" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="286" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A286" s="1" t="s">
-        <v>1291</v>
+        <v>1287</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>1292</v>
+        <v>1288</v>
       </c>
       <c r="C286" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D286" s="1" t="s">
+        <v>1289</v>
+      </c>
+      <c r="E286" s="1" t="s">
+        <v>1290</v>
+      </c>
+      <c r="F286" s="1" t="s">
+        <v>1291</v>
+      </c>
+      <c r="G286" s="1" t="s">
+        <v>1292</v>
+      </c>
+      <c r="H286" s="1" t="s">
         <v>1293</v>
       </c>
-      <c r="E286" s="1" t="s">
-        <v>1294</v>
-      </c>
-      <c r="F286" s="1" t="s">
-        <v>1295</v>
-      </c>
-      <c r="G286" s="1" t="s">
-        <v>1296</v>
-      </c>
-      <c r="H286" s="1" t="s">
-        <v>1297</v>
-      </c>
       <c r="I286" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J286" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="287" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A287" s="1" t="s">
-        <v>1298</v>
+        <v>1294</v>
       </c>
       <c r="B287" s="1" t="s">
-        <v>1299</v>
+        <v>1295</v>
       </c>
       <c r="C287" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D287" s="1" t="s">
+        <v>1296</v>
+      </c>
+      <c r="E287" s="1" t="s">
+        <v>1297</v>
+      </c>
+      <c r="F287" s="1" t="s">
+        <v>1298</v>
+      </c>
+      <c r="G287" s="1" t="s">
+        <v>1299</v>
+      </c>
+      <c r="H287" s="1" t="s">
         <v>1300</v>
       </c>
-      <c r="E287" s="1" t="s">
-        <v>1301</v>
-      </c>
-      <c r="F287" s="1" t="s">
-        <v>1302</v>
-      </c>
-      <c r="G287" s="1" t="s">
-        <v>1303</v>
-      </c>
-      <c r="H287" s="1" t="s">
-        <v>1304</v>
-      </c>
       <c r="I287" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J287" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="288" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A288" s="1" t="s">
-        <v>1305</v>
+        <v>1301</v>
       </c>
       <c r="B288" s="1" t="s">
-        <v>1306</v>
+        <v>1302</v>
       </c>
       <c r="C288" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D288" s="1" t="s">
+        <v>1303</v>
+      </c>
+      <c r="E288" s="1" t="s">
+        <v>1304</v>
+      </c>
+      <c r="F288" s="1" t="s">
+        <v>1305</v>
+      </c>
+      <c r="G288" s="1" t="s">
+        <v>1306</v>
+      </c>
+      <c r="H288" s="1" t="s">
         <v>1307</v>
       </c>
-      <c r="E288" s="1" t="s">
-        <v>1308</v>
-      </c>
-      <c r="F288" s="1" t="s">
-        <v>1309</v>
-      </c>
-      <c r="G288" s="1" t="s">
-        <v>1310</v>
-      </c>
-      <c r="H288" s="1" t="s">
-        <v>1311</v>
-      </c>
       <c r="I288" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J288" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="289" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A289" s="1" t="s">
-        <v>1312</v>
+        <v>1308</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>1313</v>
+        <v>1309</v>
       </c>
       <c r="C289" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D289" s="1" t="s">
+        <v>1310</v>
+      </c>
+      <c r="E289" s="1" t="s">
+        <v>1311</v>
+      </c>
+      <c r="F289" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="G289" s="1" t="s">
+        <v>1313</v>
+      </c>
+      <c r="H289" s="1" t="s">
         <v>1314</v>
       </c>
-      <c r="E289" s="1" t="s">
-        <v>1315</v>
-      </c>
-      <c r="F289" s="1" t="s">
-        <v>1316</v>
-      </c>
-      <c r="G289" s="1" t="s">
-        <v>1317</v>
-      </c>
-      <c r="H289" s="1" t="s">
-        <v>1318</v>
-      </c>
       <c r="I289" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J289" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="290" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A290" s="1" t="s">
-        <v>1319</v>
+        <v>1315</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>1320</v>
+        <v>1316</v>
       </c>
       <c r="C290" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D290" s="1" t="s">
+        <v>1317</v>
+      </c>
+      <c r="E290" s="1" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F290" s="1" t="s">
+        <v>1319</v>
+      </c>
+      <c r="G290" s="1" t="s">
+        <v>1320</v>
+      </c>
+      <c r="H290" s="1" t="s">
         <v>1321</v>
       </c>
-      <c r="E290" s="1" t="s">
-        <v>1322</v>
-      </c>
-      <c r="F290" s="1" t="s">
-        <v>1323</v>
-      </c>
-      <c r="G290" s="1" t="s">
-        <v>1324</v>
-      </c>
-      <c r="H290" s="1" t="s">
-        <v>1325</v>
-      </c>
       <c r="I290" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J290" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="291" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A291" s="1" t="s">
-        <v>1326</v>
+        <v>1322</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>1327</v>
+        <v>1323</v>
       </c>
       <c r="C291" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D291" s="1" t="s">
+        <v>1324</v>
+      </c>
+      <c r="E291" s="1" t="s">
+        <v>1325</v>
+      </c>
+      <c r="F291" s="1" t="s">
+        <v>1326</v>
+      </c>
+      <c r="G291" s="1" t="s">
+        <v>1327</v>
+      </c>
+      <c r="H291" s="1" t="s">
         <v>1328</v>
       </c>
-      <c r="E291" s="1" t="s">
-        <v>1329</v>
-      </c>
-      <c r="F291" s="1" t="s">
-        <v>1330</v>
-      </c>
-      <c r="G291" s="1" t="s">
-        <v>1331</v>
-      </c>
-      <c r="H291" s="1" t="s">
-        <v>1332</v>
-      </c>
       <c r="I291" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J291" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="292" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A292" s="1" t="s">
-        <v>1333</v>
+        <v>1329</v>
       </c>
       <c r="B292" s="1" t="s">
-        <v>1334</v>
+        <v>1330</v>
       </c>
       <c r="C292" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D292" s="1" t="s">
+        <v>1331</v>
+      </c>
+      <c r="E292" s="1" t="s">
+        <v>1332</v>
+      </c>
+      <c r="F292" s="1" t="s">
+        <v>1333</v>
+      </c>
+      <c r="G292" s="1" t="s">
+        <v>1334</v>
+      </c>
+      <c r="H292" s="1" t="s">
         <v>1335</v>
       </c>
-      <c r="E292" s="1" t="s">
-        <v>1336</v>
-      </c>
-      <c r="F292" s="1" t="s">
-        <v>1337</v>
-      </c>
-      <c r="G292" s="1" t="s">
-        <v>1338</v>
-      </c>
-      <c r="H292" s="1" t="s">
-        <v>1339</v>
-      </c>
       <c r="I292" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J292" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="293" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A293" s="1" t="s">
-        <v>1340</v>
+        <v>1336</v>
       </c>
       <c r="B293" s="1" t="s">
-        <v>1341</v>
+        <v>1337</v>
       </c>
       <c r="C293" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D293" s="1" t="s">
+        <v>1338</v>
+      </c>
+      <c r="E293" s="1" t="s">
+        <v>1339</v>
+      </c>
+      <c r="F293" s="1" t="s">
+        <v>1340</v>
+      </c>
+      <c r="G293" s="1" t="s">
+        <v>1341</v>
+      </c>
+      <c r="H293" s="1" t="s">
         <v>1342</v>
       </c>
-      <c r="E293" s="1" t="s">
-        <v>1343</v>
-      </c>
-      <c r="F293" s="1" t="s">
-        <v>1344</v>
-      </c>
-      <c r="G293" s="1" t="s">
-        <v>1345</v>
-      </c>
-      <c r="H293" s="1" t="s">
-        <v>1346</v>
-      </c>
       <c r="I293" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J293" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="294" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A294" s="1" t="s">
-        <v>1347</v>
+        <v>1343</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>1348</v>
+        <v>1344</v>
       </c>
       <c r="C294" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D294" s="1" t="s">
+        <v>1345</v>
+      </c>
+      <c r="E294" s="1" t="s">
+        <v>1346</v>
+      </c>
+      <c r="F294" s="1" t="s">
+        <v>1347</v>
+      </c>
+      <c r="G294" s="1" t="s">
+        <v>1348</v>
+      </c>
+      <c r="H294" s="1" t="s">
         <v>1349</v>
       </c>
-      <c r="E294" s="1" t="s">
-        <v>1350</v>
-      </c>
-      <c r="F294" s="1" t="s">
-        <v>1351</v>
-      </c>
-      <c r="G294" s="1" t="s">
-        <v>1352</v>
-      </c>
-      <c r="H294" s="1" t="s">
-        <v>1353</v>
-      </c>
       <c r="I294" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J294" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="295" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A295" s="1" t="s">
-        <v>1354</v>
+        <v>1350</v>
       </c>
       <c r="B295" s="1" t="s">
-        <v>1355</v>
+        <v>1351</v>
       </c>
       <c r="C295" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D295" s="1" t="s">
+        <v>1352</v>
+      </c>
+      <c r="E295" s="1" t="s">
+        <v>1353</v>
+      </c>
+      <c r="F295" s="1" t="s">
+        <v>1354</v>
+      </c>
+      <c r="G295" s="1" t="s">
+        <v>1355</v>
+      </c>
+      <c r="H295" s="1" t="s">
         <v>1356</v>
       </c>
-      <c r="E295" s="1" t="s">
-        <v>1357</v>
-      </c>
-      <c r="F295" s="1" t="s">
-        <v>1358</v>
-      </c>
-      <c r="G295" s="1" t="s">
-        <v>1359</v>
-      </c>
-      <c r="H295" s="1" t="s">
-        <v>1360</v>
-      </c>
       <c r="I295" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J295" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A296" s="1" t="s">
-        <v>1361</v>
+        <v>1357</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>1362</v>
+        <v>1358</v>
       </c>
       <c r="C296" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D296" s="1" t="s">
+        <v>1359</v>
+      </c>
+      <c r="E296" s="1" t="s">
+        <v>1360</v>
+      </c>
+      <c r="F296" s="1" t="s">
+        <v>1361</v>
+      </c>
+      <c r="G296" s="1" t="s">
+        <v>1362</v>
+      </c>
+      <c r="H296" s="1" t="s">
         <v>1363</v>
       </c>
-      <c r="E296" s="1" t="s">
-        <v>1364</v>
-      </c>
-      <c r="F296" s="1" t="s">
-        <v>1365</v>
-      </c>
-      <c r="G296" s="1" t="s">
-        <v>1366</v>
-      </c>
-      <c r="H296" s="1" t="s">
-        <v>1367</v>
-      </c>
       <c r="I296" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J296" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A297" s="1" t="s">
-        <v>1368</v>
+        <v>1364</v>
       </c>
       <c r="B297" s="1" t="s">
-        <v>1369</v>
+        <v>1365</v>
       </c>
       <c r="C297" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D297" s="1" t="s">
+        <v>1366</v>
+      </c>
+      <c r="E297" s="1" t="s">
+        <v>1367</v>
+      </c>
+      <c r="F297" s="1" t="s">
+        <v>1368</v>
+      </c>
+      <c r="G297" s="1" t="s">
+        <v>1369</v>
+      </c>
+      <c r="H297" s="1" t="s">
         <v>1370</v>
       </c>
-      <c r="E297" s="1" t="s">
-        <v>1371</v>
-      </c>
-      <c r="F297" s="1" t="s">
-        <v>1372</v>
-      </c>
-      <c r="G297" s="1" t="s">
-        <v>1373</v>
-      </c>
-      <c r="H297" s="1" t="s">
-        <v>1374</v>
-      </c>
       <c r="I297" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J297" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A298" s="1" t="s">
-        <v>1375</v>
+        <v>1371</v>
       </c>
       <c r="B298" s="1" t="s">
-        <v>1376</v>
+        <v>1372</v>
       </c>
       <c r="C298" s="1" t="s">
         <v>639</v>
       </c>
       <c r="D298" s="1" t="s">
+        <v>1373</v>
+      </c>
+      <c r="E298" s="1" t="s">
+        <v>1374</v>
+      </c>
+      <c r="F298" s="1" t="s">
+        <v>1375</v>
+      </c>
+      <c r="G298" s="1" t="s">
+        <v>1376</v>
+      </c>
+      <c r="H298" s="1" t="s">
         <v>1377</v>
       </c>
-      <c r="E298" s="1" t="s">
-        <v>1378</v>
-      </c>
-      <c r="F298" s="1" t="s">
-        <v>1379</v>
-      </c>
-      <c r="G298" s="1" t="s">
-        <v>1380</v>
-      </c>
-      <c r="H298" s="1" t="s">
-        <v>1381</v>
-      </c>
       <c r="I298" s="1" t="s">
-        <v>1290</v>
+        <v>1286</v>
       </c>
       <c r="J298" s="1" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>